<commit_message>
Team 작업진행중, Storage, Global 개념 추가
</commit_message>
<xml_diff>
--- a/Generated/GameData.xlsx
+++ b/Generated/GameData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/infy_mac/Unity/FactoryProject/Generated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0117BE5C-A8F2-D34E-A7ED-776B6AD14E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9052B554-0DBC-284B-94D1-8D4313069FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26600" activeTab="4" xr2:uid="{940BCB5D-19EC-984D-9BAE-40F19189B649}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="100">
   <si>
     <t>string</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -368,10 +368,6 @@
   </si>
   <si>
     <t>dropPlayerPercent</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Animal</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1307,7 +1303,7 @@
         <v>24</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1552,7 +1548,7 @@
         <v>8</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
@@ -1567,16 +1563,16 @@
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F2" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="H2" s="9"/>
       <c r="I2" s="9"/>
@@ -1592,19 +1588,19 @@
         <v>Spawner_Test</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>55</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E3" s="9">
         <v>1</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G3" s="20">
         <v>100100</v>
@@ -1806,7 +1802,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>29</v>
@@ -1857,7 +1853,7 @@
         <v>53</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>53</v>
@@ -1878,7 +1874,7 @@
         <v>21</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M3">
         <v>100</v>
@@ -1899,7 +1895,7 @@
         <v>53</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>53</v>
@@ -1920,7 +1916,7 @@
         <v>22</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M4">
         <v>100</v>
@@ -1941,7 +1937,7 @@
         <v>53</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>53</v>
@@ -1962,7 +1958,7 @@
         <v>22</v>
       </c>
       <c r="L5" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M5">
         <v>100</v>
@@ -1983,7 +1979,7 @@
         <v>53</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>53</v>
@@ -2004,7 +2000,7 @@
         <v>22</v>
       </c>
       <c r="L6" s="19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="M6">
         <v>100</v>
@@ -2311,7 +2307,7 @@
         <v>9</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O2" s="6"/>
       <c r="P2" s="6"/>
@@ -2474,7 +2470,7 @@
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="18" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>22</v>
@@ -2517,7 +2513,7 @@
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="18" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>22</v>
@@ -2560,7 +2556,7 @@
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="18" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>22</v>
@@ -2603,7 +2599,7 @@
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="18" t="s">
-        <v>83</v>
+        <v>7</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
Player Follow 기능 추가
</commit_message>
<xml_diff>
--- a/Generated/GameData.xlsx
+++ b/Generated/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/infy_mac/Unity/FactoryProject/Generated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16015290-64A9-1F49-8CC1-419FF8348147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB1D79F0-AEDD-6F46-B6D1-8F5F7CED4291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51160" yWindow="1100" windowWidth="51200" windowHeight="26600" activeTab="3" xr2:uid="{940BCB5D-19EC-984D-9BAE-40F19189B649}"/>
+    <workbookView xWindow="51160" yWindow="1100" windowWidth="51200" windowHeight="26600" activeTab="5" xr2:uid="{940BCB5D-19EC-984D-9BAE-40F19189B649}"/>
   </bookViews>
   <sheets>
     <sheet name="Enum" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="113">
   <si>
     <t>string</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -674,7 +674,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -733,6 +733,12 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2785,25 +2791,27 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{791254EB-5610-D14F-ACAF-D2B5E0C5153F}">
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:17">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>101</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>110</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>2</v>
@@ -2817,22 +2825,26 @@
       <c r="H1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
+      <c r="I1" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="K1" s="8"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
       <c r="N1" s="5"/>
       <c r="O1" s="5"/>
-    </row>
-    <row r="2" spans="1:15">
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="8"/>
+      <c r="D2" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>108</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>112</v>
@@ -2847,27 +2859,27 @@
         <v>103</v>
       </c>
       <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
+      <c r="J2" s="6" t="s">
+        <v>108</v>
+      </c>
       <c r="K2" s="8"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
       <c r="N2" s="6"/>
       <c r="O2" s="6"/>
-    </row>
-    <row r="3" spans="1:15">
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="7" t="str">
-        <f>_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
+        <f>_xlfn.TEXTJOIN("_",TRUE,B3,D3)</f>
         <v>FactionRelation_Hero</v>
       </c>
       <c r="B3" t="s">
         <v>109</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>112</v>
-      </c>
-      <c r="D3" s="9" t="str">
-        <f>_xlfn.TEXTJOIN(",",TRUE,E3:O3)</f>
-        <v>Friendly,Hostile,Hostile,Hostile</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>107</v>
@@ -2881,25 +2893,26 @@
       <c r="H3" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="I3" s="15"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="15"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="9" t="str">
+        <f>_xlfn.TEXTJOIN(",",TRUE,E3:H3)</f>
+        <v>Friendly,Hostile,Hostile,Hostile</v>
+      </c>
+      <c r="K3" s="9"/>
       <c r="L3" s="15"/>
-    </row>
-    <row r="4" spans="1:15">
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="7" t="str">
-        <f>_xlfn.TEXTJOIN("_",TRUE,B4,C4)</f>
+        <f>_xlfn.TEXTJOIN("_",TRUE,B4,D4)</f>
         <v>FactionRelation_Faction2</v>
       </c>
       <c r="B4" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>104</v>
-      </c>
-      <c r="D4" s="9" t="str">
-        <f>_xlfn.TEXTJOIN(",",TRUE,E4:O4)</f>
-        <v>Hostile,Friendly,Hostile,Hostile</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>105</v>
@@ -2913,25 +2926,26 @@
       <c r="H4" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="I4" s="15"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="15"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="9" t="str">
+        <f>_xlfn.TEXTJOIN(",",TRUE,E4:H4)</f>
+        <v>Hostile,Friendly,Hostile,Hostile</v>
+      </c>
+      <c r="K4" s="9"/>
       <c r="L4" s="15"/>
-    </row>
-    <row r="5" spans="1:15">
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="7" t="str">
-        <f>_xlfn.TEXTJOIN("_",TRUE,B5,C5)</f>
+        <f>_xlfn.TEXTJOIN("_",TRUE,B5,D5)</f>
         <v>FactionRelation_Faction3</v>
       </c>
       <c r="B5" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="D5" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="D5" s="9" t="str">
-        <f>_xlfn.TEXTJOIN(",",TRUE,E5:O5)</f>
-        <v>Hostile,Hostile,Friendly,Hostile</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>105</v>
@@ -2945,25 +2959,26 @@
       <c r="H5" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="I5" s="15"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="15"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="9" t="str">
+        <f>_xlfn.TEXTJOIN(",",TRUE,E5:H5)</f>
+        <v>Hostile,Hostile,Friendly,Hostile</v>
+      </c>
+      <c r="K5" s="9"/>
       <c r="L5" s="15"/>
-    </row>
-    <row r="6" spans="1:15">
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="7" t="str">
-        <f>_xlfn.TEXTJOIN("_",TRUE,B6,C6)</f>
+        <f>_xlfn.TEXTJOIN("_",TRUE,B6,D6)</f>
         <v>FactionRelation_Faction4</v>
       </c>
       <c r="B6" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="D6" s="9" t="s">
         <v>103</v>
-      </c>
-      <c r="D6" s="9" t="str">
-        <f>_xlfn.TEXTJOIN(",",TRUE,E6:O6)</f>
-        <v>Hostile,Hostile,Hostile,Friendly</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>105</v>
@@ -2977,70 +2992,81 @@
       <c r="H6" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="I6" s="9"/>
-    </row>
-    <row r="7" spans="1:15">
-      <c r="C7" s="9"/>
-      <c r="D7" s="18"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="9" t="str">
+        <f>_xlfn.TEXTJOIN(",",TRUE,E6:H6)</f>
+        <v>Hostile,Hostile,Hostile,Friendly</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
+      <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
       <c r="I7" s="15"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="15"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="9"/>
       <c r="L7" s="15"/>
-    </row>
-    <row r="8" spans="1:15">
-      <c r="C8" s="9"/>
-      <c r="D8" s="18"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+    </row>
+    <row r="8" spans="1:17">
+      <c r="D8" s="9"/>
       <c r="E8" s="9"/>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
       <c r="H8" s="15"/>
       <c r="I8" s="15"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="15"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="9"/>
       <c r="L8" s="15"/>
-    </row>
-    <row r="9" spans="1:15">
-      <c r="C9" s="9"/>
-      <c r="D9" s="18"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+    </row>
+    <row r="9" spans="1:17">
+      <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="15"/>
       <c r="G9" s="15"/>
       <c r="H9" s="15"/>
       <c r="I9" s="15"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="15"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="9"/>
       <c r="L9" s="15"/>
-    </row>
-    <row r="10" spans="1:15">
-      <c r="C10" s="9"/>
-      <c r="D10" s="18"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+    </row>
+    <row r="10" spans="1:17">
+      <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="15"/>
       <c r="G10" s="15"/>
       <c r="H10" s="15"/>
       <c r="I10" s="15"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="15"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="9"/>
       <c r="L10" s="15"/>
-    </row>
-    <row r="11" spans="1:15">
-      <c r="C11" s="9"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+    </row>
+    <row r="11" spans="1:17">
       <c r="D11" s="9"/>
       <c r="H11" s="9"/>
-    </row>
-    <row r="12" spans="1:15">
-      <c r="C12" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+    </row>
+    <row r="12" spans="1:17">
       <c r="D12" s="9"/>
       <c r="H12" s="9"/>
-    </row>
-    <row r="13" spans="1:15">
-      <c r="C13" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+    </row>
+    <row r="13" spans="1:17">
       <c r="D13" s="9"/>
       <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -3052,7 +3078,7 @@
           <x14:formula1>
             <xm:f>Enum!$H$2:$H$1013</xm:f>
           </x14:formula1>
-          <xm:sqref>K6 O3:O7</xm:sqref>
+          <xm:sqref>L6:M6 Q3:Q7</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Constant 추가, Flow 임시데이터 설정, BrainAbility 수정, SearchLogic 추가
</commit_message>
<xml_diff>
--- a/Generated/GameData.xlsx
+++ b/Generated/GameData.xlsx
@@ -1,42 +1,53 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Toy\Project\FactoryProject\Generated\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/infy_mac/Unity/FactoryProject/Generated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0206A45-9534-49AC-9AFE-D1FA6DCADE56}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F249AE7-7F29-B742-9C37-4A6A19CF14BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="500" windowWidth="51200" windowHeight="26600" activeTab="9" xr2:uid="{940BCB5D-19EC-984D-9BAE-40F19189B649}"/>
+    <workbookView xWindow="51180" yWindow="500" windowWidth="51200" windowHeight="26600" activeTab="10" xr2:uid="{940BCB5D-19EC-984D-9BAE-40F19189B649}"/>
   </bookViews>
   <sheets>
     <sheet name="Enum" sheetId="2" r:id="rId1"/>
-    <sheet name="Localization" sheetId="8" r:id="rId2"/>
-    <sheet name="Spawner" sheetId="23" r:id="rId3"/>
-    <sheet name="Player" sheetId="4" r:id="rId4"/>
-    <sheet name="Item" sheetId="19" r:id="rId5"/>
-    <sheet name="FactionRelation" sheetId="24" r:id="rId6"/>
-    <sheet name="Grade" sheetId="22" r:id="rId7"/>
-    <sheet name="SynergeBiome" sheetId="20" r:id="rId8"/>
-    <sheet name="SynergeElement" sheetId="21" r:id="rId9"/>
-    <sheet name="Skill" sheetId="27" r:id="rId10"/>
-    <sheet name="Buff" sheetId="29" r:id="rId11"/>
-    <sheet name="Projectile" sheetId="28" r:id="rId12"/>
+    <sheet name="Constant" sheetId="30" r:id="rId2"/>
+    <sheet name="Localization" sheetId="8" r:id="rId3"/>
+    <sheet name="Spawner" sheetId="23" r:id="rId4"/>
+    <sheet name="Player" sheetId="4" r:id="rId5"/>
+    <sheet name="Item" sheetId="19" r:id="rId6"/>
+    <sheet name="FactionRelation" sheetId="24" r:id="rId7"/>
+    <sheet name="Grade" sheetId="22" r:id="rId8"/>
+    <sheet name="SynergeBiome" sheetId="20" r:id="rId9"/>
+    <sheet name="SynergeElement" sheetId="21" r:id="rId10"/>
+    <sheet name="Skill" sheetId="27" r:id="rId11"/>
+    <sheet name="Buff" sheetId="29" r:id="rId12"/>
+    <sheet name="Projectile" sheetId="28" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="190">
   <si>
     <t>string</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -730,6 +741,66 @@
   </si>
   <si>
     <t>cooldown</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>rawValue</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DataType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>String</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Float</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Long</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dataType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DefaultDetectionRange</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Flow</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DefaultAttackRange</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TargetLostRangeOffset</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FoolowDistanceRatio</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>// AI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>hp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>: Str * 100</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -737,7 +808,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -915,7 +986,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -970,9 +1041,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1290,13 +1358,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD4AE1AA-8A06-FD4D-90BD-9F8B147AB8E0}">
   <dimension ref="A1:S70"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
-    <col min="2" max="2" width="13.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:19">
       <c r="A1" s="1">
         <v>1</v>
       </c>
@@ -1319,7 +1387,7 @@
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:19">
       <c r="A2" s="1">
         <v>2</v>
       </c>
@@ -1330,7 +1398,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:19">
       <c r="A3" s="1">
         <v>3</v>
       </c>
@@ -1341,7 +1409,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:19">
       <c r="A4" s="1">
         <v>4</v>
       </c>
@@ -1352,7 +1420,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:19">
       <c r="A5" s="1">
         <v>5</v>
       </c>
@@ -1363,7 +1431,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:19">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -1374,7 +1442,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:19">
       <c r="A7" s="1">
         <v>2</v>
       </c>
@@ -1385,7 +1453,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:19">
       <c r="A8" s="1">
         <v>3</v>
       </c>
@@ -1396,7 +1464,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:19">
       <c r="A9" s="1">
         <v>4</v>
       </c>
@@ -1407,7 +1475,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:19">
       <c r="A10" s="1">
         <v>5</v>
       </c>
@@ -1418,7 +1486,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:19">
       <c r="A11" s="1">
         <v>6</v>
       </c>
@@ -1429,7 +1497,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:19">
       <c r="A12" s="1">
         <v>1</v>
       </c>
@@ -1440,7 +1508,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:19">
       <c r="A13" s="1">
         <v>2</v>
       </c>
@@ -1451,7 +1519,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:19">
       <c r="A14" s="1">
         <v>3</v>
       </c>
@@ -1462,7 +1530,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:19">
       <c r="A15" s="1">
         <v>4</v>
       </c>
@@ -1473,7 +1541,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:19">
       <c r="A16" s="1">
         <v>5</v>
       </c>
@@ -1484,7 +1552,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5">
       <c r="A17" s="1">
         <v>6</v>
       </c>
@@ -1495,7 +1563,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5">
       <c r="A18" s="1">
         <v>7</v>
       </c>
@@ -1506,7 +1574,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5">
       <c r="A19" s="1">
         <v>8</v>
       </c>
@@ -1517,7 +1585,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -1528,7 +1596,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5">
       <c r="A21" s="1">
         <v>2</v>
       </c>
@@ -1540,7 +1608,7 @@
       </c>
       <c r="E21" s="11"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5">
       <c r="A22" s="1">
         <v>3</v>
       </c>
@@ -1552,7 +1620,7 @@
       </c>
       <c r="E22" s="11"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:5">
       <c r="A23" s="1">
         <v>4</v>
       </c>
@@ -1564,7 +1632,7 @@
       </c>
       <c r="E23" s="11"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:5">
       <c r="A24" s="1">
         <v>1</v>
       </c>
@@ -1576,7 +1644,7 @@
       </c>
       <c r="E24" s="11"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5">
       <c r="A25" s="1">
         <v>2</v>
       </c>
@@ -1588,7 +1656,7 @@
       </c>
       <c r="E25" s="11"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5">
       <c r="A26" s="1">
         <v>3</v>
       </c>
@@ -1600,7 +1668,7 @@
       </c>
       <c r="E26" s="12"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5">
       <c r="A27" s="1">
         <v>4</v>
       </c>
@@ -1611,7 +1679,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5">
       <c r="A28" s="1">
         <v>5</v>
       </c>
@@ -1622,7 +1690,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5">
       <c r="A29" s="1">
         <v>1</v>
       </c>
@@ -1633,7 +1701,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5">
       <c r="A30" s="1">
         <v>2</v>
       </c>
@@ -1644,7 +1712,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:5">
       <c r="A31" s="1">
         <v>3</v>
       </c>
@@ -1655,7 +1723,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:5">
       <c r="A32" s="1">
         <v>1</v>
       </c>
@@ -1666,7 +1734,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:11">
       <c r="A33" s="1">
         <v>2</v>
       </c>
@@ -1677,7 +1745,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:11">
       <c r="A34" s="1">
         <v>3</v>
       </c>
@@ -1688,7 +1756,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:11">
       <c r="A35" s="1">
         <v>4</v>
       </c>
@@ -1699,7 +1767,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:11">
       <c r="A36" s="1">
         <v>1</v>
       </c>
@@ -1710,7 +1778,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:11">
       <c r="A37" s="1">
         <v>2</v>
       </c>
@@ -1721,7 +1789,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:11">
       <c r="A38" s="1">
         <v>1</v>
       </c>
@@ -1732,7 +1800,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:11">
       <c r="A39" s="1">
         <v>2</v>
       </c>
@@ -1743,7 +1811,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:11">
       <c r="A40" s="1">
         <v>1</v>
       </c>
@@ -1754,7 +1822,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:11">
       <c r="A41" s="1">
         <v>2</v>
       </c>
@@ -1765,7 +1833,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:11">
       <c r="A42" s="1">
         <v>3</v>
       </c>
@@ -1776,7 +1844,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:11">
       <c r="A43" s="1">
         <v>4</v>
       </c>
@@ -1791,7 +1859,7 @@
       <c r="J43" s="11"/>
       <c r="K43" s="11"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:11">
       <c r="A44" s="1">
         <v>5</v>
       </c>
@@ -1805,7 +1873,7 @@
       <c r="J44" s="11"/>
       <c r="K44" s="11"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:11">
       <c r="A45" s="1">
         <v>6</v>
       </c>
@@ -1816,7 +1884,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:11">
       <c r="A46" s="1">
         <v>1</v>
       </c>
@@ -1827,7 +1895,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:11">
       <c r="A47" s="1">
         <v>2</v>
       </c>
@@ -1838,7 +1906,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:11">
       <c r="A48" s="1">
         <v>3</v>
       </c>
@@ -1849,99 +1917,123 @@
         <v>165</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A49" s="1"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="1"/>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A50" s="1"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="1"/>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A51" s="1"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="1"/>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A52" s="1"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="1"/>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:3">
+      <c r="A49" s="1">
+        <v>1</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="1">
+        <v>2</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" s="1">
+        <v>3</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="1">
+        <v>4</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
       <c r="A53" s="1"/>
       <c r="B53" s="11"/>
       <c r="C53" s="1"/>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:3">
       <c r="A54" s="1"/>
       <c r="B54" s="11"/>
       <c r="C54" s="1"/>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:3">
       <c r="A55" s="1"/>
       <c r="B55" s="11"/>
       <c r="C55" s="1"/>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:3">
       <c r="A56" s="1"/>
       <c r="B56" s="11"/>
       <c r="C56" s="1"/>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:3">
       <c r="A57" s="1"/>
       <c r="C57" s="1"/>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:3">
       <c r="A58" s="1"/>
       <c r="C58" s="1"/>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:3">
       <c r="A59" s="1"/>
       <c r="C59" s="1"/>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:3">
       <c r="A60" s="1"/>
       <c r="C60" s="1"/>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:3">
       <c r="A61" s="1"/>
       <c r="C61" s="1"/>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:3">
       <c r="A62" s="1"/>
       <c r="C62" s="1"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:3">
       <c r="A63" s="1"/>
       <c r="C63" s="1"/>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:3">
       <c r="A64" s="1"/>
       <c r="C64" s="1"/>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:3">
       <c r="A65" s="1"/>
       <c r="C65" s="1"/>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:3">
       <c r="A66" s="1"/>
       <c r="C66" s="1"/>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:3">
       <c r="A67" s="1"/>
       <c r="C67" s="1"/>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:3">
       <c r="A68" s="1"/>
       <c r="C68" s="1"/>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:3">
       <c r="A69" s="1"/>
       <c r="C69" s="1"/>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:3">
       <c r="A70" s="1"/>
     </row>
   </sheetData>
@@ -1957,22 +2049,114 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E95C1629-BD9D-564A-BFD4-EB36E5A37A98}">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="7"/>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="7" t="str">
+        <f>_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
+        <v>SynergeElement_Test</v>
+      </c>
+      <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="C4" s="9"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="C5" s="9"/>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="C6" s="9"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B5FDDF60-689E-184E-934A-907BC1C56072}">
+          <x14:formula1>
+            <xm:f>Enum!$I$2:$I$1017</xm:f>
+          </x14:formula1>
+          <xm:sqref>B5:B6</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4766A74-1CE1-8948-A88A-472E2BC79D97}">
   <dimension ref="A1:AF19"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="23.3046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.53515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.15234375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="19.3046875" customWidth="1"/>
-    <col min="13" max="13" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.84375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.53515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="19.28515625" customWidth="1"/>
+    <col min="13" max="13" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:32">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -1989,7 +2173,7 @@
       <c r="F1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="19" t="s">
         <v>173</v>
       </c>
       <c r="H1" s="19" t="s">
@@ -2036,14 +2220,14 @@
       <c r="AE1" s="5"/>
       <c r="AF1" s="5"/>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:32">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
-      <c r="G2" s="20" t="s">
+      <c r="G2" s="19" t="s">
         <v>174</v>
       </c>
       <c r="H2" s="19" t="s">
@@ -2090,7 +2274,7 @@
       <c r="AE2" s="6"/>
       <c r="AF2" s="6"/>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:32">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -2115,28 +2299,28 @@
       <c r="Q3" s="9"/>
       <c r="S3" s="9"/>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:32">
       <c r="A4" s="7" t="s">
         <v>2</v>
       </c>
       <c r="S4" s="13"/>
       <c r="T4" s="1"/>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:32">
       <c r="A5" s="7" t="s">
         <v>152</v>
       </c>
       <c r="S5" s="13"/>
       <c r="T5" s="1"/>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:32">
       <c r="A6" s="7" t="s">
         <v>152</v>
       </c>
       <c r="S6" s="13"/>
       <c r="T6" s="1"/>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:32">
       <c r="A7" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B7:F7)</f>
         <v>Skill_Human_Projectile_1</v>
@@ -2182,26 +2366,26 @@
       <c r="S7" s="13"/>
       <c r="T7" s="1"/>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:32">
       <c r="A8" s="7" t="s">
         <v>2</v>
       </c>
       <c r="S8" s="13"/>
       <c r="T8" s="1"/>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:32">
       <c r="A9" s="7" t="s">
         <v>153</v>
       </c>
       <c r="S9" s="13"/>
       <c r="T9" s="1"/>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:32">
       <c r="A10" s="7" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:32">
       <c r="A11" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B11:F11)</f>
         <v>Skill_Projectile_Hit_1</v>
@@ -2244,11 +2428,11 @@
       <c r="O11" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="P11" s="11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.45">
+      <c r="P11" s="11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32">
       <c r="A12" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B12:F12)</f>
         <v>Skill_Human_MeleeAttack_1</v>
@@ -2290,26 +2474,26 @@
       <c r="O12" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="P12" s="11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.45">
+      <c r="P12" s="11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="13" spans="1:32">
       <c r="A13" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:32">
       <c r="A14" s="7" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:32">
       <c r="A15" s="7" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:32">
       <c r="A16" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B16:F16)</f>
         <v>Skill_Stat_1</v>
@@ -2354,12 +2538,12 @@
         <v>162</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:16">
       <c r="A18" s="19" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:16">
       <c r="A19" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B19:F19)</f>
         <v>Skill_Human_AddBuff_1</v>
@@ -2418,19 +2602,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38C8E724-28BD-8649-A64E-E00F04A859F7}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="15.3828125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.84375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.15234375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.3828125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:12">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -2466,7 +2650,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
@@ -2494,7 +2678,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12">
       <c r="A3" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B3:E3)</f>
         <v>Buff_1</v>
@@ -2529,7 +2713,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12">
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2539,20 +2723,20 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12">
       <c r="F6" s="9"/>
       <c r="G6" s="9"/>
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
       <c r="J6" s="9"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12">
       <c r="G7" s="9"/>
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12">
       <c r="F8" s="9"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9"/>
@@ -2566,21 +2750,21 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7280A486-F06C-3245-9C19-439155A4666B}">
   <dimension ref="A1:O7"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="15.3828125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.84375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.15234375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.3828125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.3046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.53515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:15">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -2611,7 +2795,7 @@
       <c r="N1" s="9"/>
       <c r="O1" s="11"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:15">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
@@ -2638,7 +2822,7 @@
       <c r="N2" s="9"/>
       <c r="O2" s="11"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15">
       <c r="A3" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
         <v>Projectile_Human</v>
@@ -2672,7 +2856,7 @@
       <c r="N3" s="9"/>
       <c r="O3" s="11"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:15">
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2687,7 +2871,7 @@
       <c r="N4" s="9"/>
       <c r="O4" s="11"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15">
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -2702,7 +2886,7 @@
       <c r="N5" s="9"/>
       <c r="O5" s="11"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:15">
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -2717,7 +2901,7 @@
       <c r="N6" s="9"/>
       <c r="O6" s="11"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:15">
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
@@ -2736,34 +2920,181 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{375CF63E-9079-1A4A-A3AF-0BA8892B823F}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="20.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="7"/>
+      <c r="B1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="9"/>
+      <c r="G3" s="9"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="7" t="str">
+        <f>_xlfn.TEXTJOIN("_",TRUE,B5:D5)</f>
+        <v>AI_Flow_DefaultDetectionRange</v>
+      </c>
+      <c r="B5" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="9"/>
+      <c r="F5" t="s">
+        <v>178</v>
+      </c>
+      <c r="G5" s="9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="7" t="str">
+        <f t="shared" ref="A6:A8" si="0">_xlfn.TEXTJOIN("_",TRUE,B6:D6)</f>
+        <v>AI_Flow_DefaultAttackRange</v>
+      </c>
+      <c r="B6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D6" t="s">
+        <v>184</v>
+      </c>
+      <c r="F6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G6" s="9">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>AI_Flow_TargetLostRangeOffset</v>
+      </c>
+      <c r="B7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" t="s">
+        <v>183</v>
+      </c>
+      <c r="D7" t="s">
+        <v>185</v>
+      </c>
+      <c r="F7" t="s">
+        <v>178</v>
+      </c>
+      <c r="G7" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="7" t="str">
+        <f t="shared" si="0"/>
+        <v>AI_Flow_FoolowDistanceRatio</v>
+      </c>
+      <c r="B8" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" t="s">
+        <v>183</v>
+      </c>
+      <c r="D8" t="s">
+        <v>186</v>
+      </c>
+      <c r="F8" t="s">
+        <v>178</v>
+      </c>
+      <c r="G8" s="9">
+        <v>0.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9012A38-B8D5-894C-A1D0-EDAD32738ED4}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7454E3B-BCDE-5A49-BB39-4B30666D97F3}">
   <dimension ref="A1:P12"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
-    <col min="4" max="4" width="19.15234375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.15234375" customWidth="1"/>
-    <col min="6" max="6" width="20.69140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.3046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.84375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.3046875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.15234375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.53515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.84375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:16">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -2791,7 +3122,7 @@
       <c r="M1" s="9"/>
       <c r="N1" s="11"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:16">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
@@ -2815,7 +3146,7 @@
       <c r="M2" s="9"/>
       <c r="N2" s="11"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:16">
       <c r="A3" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
         <v>Spawner_Test</v>
@@ -2846,7 +3177,7 @@
       <c r="M3" s="9"/>
       <c r="N3" s="11"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:16">
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -2860,7 +3191,7 @@
       <c r="M4" s="9"/>
       <c r="N4" s="11"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:16">
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -2874,7 +3205,7 @@
       <c r="M5" s="9"/>
       <c r="N5" s="11"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:16">
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -2890,7 +3221,7 @@
       <c r="O6" s="9"/>
       <c r="P6" s="11"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:16">
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
@@ -2906,7 +3237,7 @@
       <c r="O7" s="9"/>
       <c r="P7" s="11"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:16">
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
@@ -2920,7 +3251,7 @@
       <c r="M8" s="9"/>
       <c r="N8" s="11"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:16">
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
@@ -2934,7 +3265,7 @@
       <c r="M9" s="9"/>
       <c r="N9" s="11"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:16">
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
@@ -2943,7 +3274,7 @@
       <c r="H10" s="9"/>
       <c r="L10" s="9"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:16">
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
@@ -2952,7 +3283,7 @@
       <c r="H11" s="9"/>
       <c r="L11" s="9"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:16">
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
@@ -2967,29 +3298,29 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A933480A-994B-A74A-B07D-EEB09A80B87F}">
-  <dimension ref="A1:V32"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:W32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.15234375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.53515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.3828125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="21.69140625" customWidth="1"/>
-    <col min="12" max="12" width="21.69140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.84375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="21.7109375" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:23">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="5"/>
       <c r="D1" s="5" t="s">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>0</v>
@@ -3000,91 +3331,97 @@
       <c r="G1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="K1" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="Q1" s="5"/>
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
       <c r="T1" s="5"/>
       <c r="U1" s="5"/>
       <c r="V1" s="5"/>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="W1" s="5"/>
+    </row>
+    <row r="2" spans="1:23">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="16" t="s">
+      <c r="K2" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="M2" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="O2" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="P2" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="Q2" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="14"/>
       <c r="T2" s="6"/>
       <c r="U2" s="6"/>
       <c r="V2" s="6"/>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="W2" s="6"/>
+    </row>
+    <row r="3" spans="1:23">
       <c r="A3" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
         <v>Player_Human</v>
@@ -3095,44 +3432,47 @@
       <c r="C3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="9">
+        <v>100</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="I3" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="J3" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="K3" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="L3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="11" t="s">
+      <c r="M3" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="M3" s="9">
+      <c r="N3" s="9">
         <v>100</v>
       </c>
-      <c r="N3" s="11" t="s">
+      <c r="O3" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:23">
       <c r="A4" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B4,C4)</f>
         <v>Player_Dog</v>
@@ -3143,44 +3483,47 @@
       <c r="C4" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="9">
+        <v>100</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="I4" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="I4" s="11" t="s">
+      <c r="J4" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="K4" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="L4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="11" t="s">
+      <c r="M4" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="M4" s="9">
+      <c r="N4" s="9">
         <v>100</v>
       </c>
-      <c r="N4" s="11" t="s">
+      <c r="O4" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:23">
       <c r="A5" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B5,C5)</f>
         <v>Player_Eagle</v>
@@ -3191,44 +3534,47 @@
       <c r="C5" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="9">
+        <v>100</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="H5" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="J5" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="K5" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="K5" s="9" t="s">
+      <c r="L5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="11" t="s">
+      <c r="M5" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="M5" s="9">
+      <c r="N5" s="9">
         <v>100</v>
       </c>
-      <c r="N5" s="11" t="s">
+      <c r="O5" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:23">
       <c r="A6" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B6,C6)</f>
         <v>Player_Snake</v>
@@ -3239,44 +3585,47 @@
       <c r="C6" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="9">
+        <v>100</v>
+      </c>
+      <c r="E6" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="I6" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="J6" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="K6" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="K6" s="9" t="s">
+      <c r="L6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="11" t="s">
+      <c r="M6" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="M6" s="9">
+      <c r="N6" s="9">
         <v>100</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="O6" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:23">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -3285,190 +3634,216 @@
       <c r="E7" s="9"/>
       <c r="F7" s="9"/>
       <c r="G7" s="9"/>
-      <c r="H7" s="11"/>
+      <c r="H7" s="9"/>
       <c r="I7" s="11"/>
       <c r="J7" s="11"/>
-      <c r="K7" s="9"/>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="K7" s="11"/>
+      <c r="L7" s="9"/>
+    </row>
+    <row r="8" spans="1:23">
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
       <c r="F8" s="9"/>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="G8" s="9"/>
+      <c r="K8" s="9"/>
+    </row>
+    <row r="9" spans="1:23">
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="G9" s="9"/>
+      <c r="K9" s="9"/>
+    </row>
+    <row r="10" spans="1:23">
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
-      <c r="J10" s="9"/>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="G10" s="9"/>
+      <c r="K10" s="9"/>
+    </row>
+    <row r="11" spans="1:23">
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="F11" s="9"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="G11" s="9"/>
+      <c r="K11" s="9"/>
+    </row>
+    <row r="12" spans="1:23">
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
-      <c r="G12" s="4"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="G12" s="9"/>
+      <c r="H12" s="4"/>
+      <c r="K12" s="9"/>
+    </row>
+    <row r="13" spans="1:23">
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="G13" s="9"/>
+      <c r="K13" s="9"/>
+    </row>
+    <row r="14" spans="1:23">
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="9"/>
       <c r="F14" s="9"/>
-      <c r="G14" s="3"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="G14" s="9"/>
+      <c r="H14" s="3"/>
+      <c r="K14" s="9"/>
+    </row>
+    <row r="15" spans="1:23">
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
-      <c r="G15" s="4"/>
-      <c r="J15" s="9"/>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="G15" s="9"/>
+      <c r="H15" s="4"/>
+      <c r="K15" s="9"/>
+    </row>
+    <row r="16" spans="1:23">
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="4"/>
-      <c r="J16" s="9"/>
-    </row>
-    <row r="17" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G16" s="9"/>
+      <c r="H16" s="4"/>
+      <c r="K16" s="9"/>
+    </row>
+    <row r="17" spans="3:11">
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
-      <c r="J17" s="9"/>
-    </row>
-    <row r="18" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="H17" s="9"/>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="18" spans="3:11">
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
-      <c r="J18" s="9"/>
-    </row>
-    <row r="19" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G18" s="9"/>
+      <c r="K18" s="9"/>
+    </row>
+    <row r="19" spans="3:11">
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
-      <c r="J19" s="9"/>
-    </row>
-    <row r="20" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G19" s="9"/>
+      <c r="K19" s="9"/>
+    </row>
+    <row r="20" spans="3:11">
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
-      <c r="J20" s="9"/>
-    </row>
-    <row r="21" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G20" s="9"/>
+      <c r="K20" s="9"/>
+    </row>
+    <row r="21" spans="3:11">
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
       <c r="E21" s="9"/>
       <c r="F21" s="9"/>
-      <c r="J21" s="9"/>
-    </row>
-    <row r="22" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G21" s="9"/>
+      <c r="K21" s="9"/>
+    </row>
+    <row r="22" spans="3:11">
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
-      <c r="J22" s="9"/>
-    </row>
-    <row r="23" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G22" s="9"/>
+      <c r="K22" s="9"/>
+    </row>
+    <row r="23" spans="3:11">
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
       <c r="F23" s="9"/>
-      <c r="J23" s="9"/>
-    </row>
-    <row r="24" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G23" s="9"/>
+      <c r="K23" s="9"/>
+    </row>
+    <row r="24" spans="3:11">
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
-      <c r="J24" s="9"/>
-    </row>
-    <row r="25" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G24" s="9"/>
+      <c r="K24" s="9"/>
+    </row>
+    <row r="25" spans="3:11">
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
-      <c r="J25" s="9"/>
-    </row>
-    <row r="26" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G25" s="9"/>
+      <c r="K25" s="9"/>
+    </row>
+    <row r="26" spans="3:11">
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
-      <c r="J26" s="9"/>
-    </row>
-    <row r="27" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G26" s="9"/>
+      <c r="K26" s="9"/>
+    </row>
+    <row r="27" spans="3:11">
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
-      <c r="J27" s="9"/>
-    </row>
-    <row r="28" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G27" s="9"/>
+      <c r="K27" s="9"/>
+    </row>
+    <row r="28" spans="3:11">
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
       <c r="F28" s="9"/>
-      <c r="J28" s="9"/>
-    </row>
-    <row r="29" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G28" s="9"/>
+      <c r="K28" s="9"/>
+    </row>
+    <row r="29" spans="3:11">
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="9"/>
-      <c r="J29" s="9"/>
-    </row>
-    <row r="30" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G29" s="9"/>
+      <c r="K29" s="9"/>
+    </row>
+    <row r="30" spans="3:11">
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
       <c r="F30" s="9"/>
-      <c r="J30" s="9"/>
-    </row>
-    <row r="31" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G30" s="9"/>
+      <c r="K30" s="9"/>
+    </row>
+    <row r="31" spans="3:11">
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="9"/>
-      <c r="J31" s="9"/>
-    </row>
-    <row r="32" spans="3:10" x14ac:dyDescent="0.45">
+      <c r="G31" s="9"/>
+      <c r="K31" s="9"/>
+    </row>
+    <row r="32" spans="3:11">
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
       <c r="F32" s="9"/>
-      <c r="J32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="K32" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -3480,7 +3855,7 @@
           <x14:formula1>
             <xm:f>Enum!$H$2:$H$1017</xm:f>
           </x14:formula1>
-          <xm:sqref>Q3:Q7</xm:sqref>
+          <xm:sqref>R3:R7</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3488,18 +3863,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AA670E5-D6A8-8742-AF98-6CB0AA05A8B1}">
   <dimension ref="A1:V14"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="15.53515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.15234375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.3046875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:22">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -3547,7 +3922,7 @@
       <c r="U1" s="5"/>
       <c r="V1" s="5"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:22">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
@@ -3589,7 +3964,7 @@
       <c r="U2" s="6"/>
       <c r="V2" s="6"/>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:22">
       <c r="A3" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
         <v>Item_WoodSword</v>
@@ -3629,7 +4004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:22">
       <c r="A4" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B4,C4)</f>
         <v>Item_WoodStaff</v>
@@ -3669,7 +4044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:22">
       <c r="A5" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B5,C5)</f>
         <v>Item_WoodBow</v>
@@ -3709,7 +4084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:22">
       <c r="A6" s="7" t="s">
         <v>2</v>
       </c>
@@ -3719,7 +4094,7 @@
       <c r="I6" s="11"/>
       <c r="J6" s="11"/>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:22">
       <c r="A7" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B7,C7)</f>
         <v>Item_Human</v>
@@ -3759,7 +4134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:22">
       <c r="A8" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B8,C8)</f>
         <v>Item_Dog</v>
@@ -3799,7 +4174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:22">
       <c r="A9" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B9,C9)</f>
         <v>Item_Eagle</v>
@@ -3839,7 +4214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:22">
       <c r="A10" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B10,C10)</f>
         <v>Item_Snake</v>
@@ -3879,25 +4254,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:22">
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="E11" s="9"/>
       <c r="I11" s="9"/>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:22">
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="I12" s="9"/>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:22">
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="E13" s="9"/>
       <c r="I13" s="1"/>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:22">
       <c r="I14" s="1"/>
     </row>
   </sheetData>
@@ -3923,20 +4298,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{791254EB-5610-D14F-ACAF-D2B5E0C5153F}">
   <dimension ref="A1:Q13"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="21.53515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.53515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.53515625" customWidth="1"/>
-    <col min="4" max="4" width="10.84375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.3046875" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="26.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:17">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -3973,7 +4348,7 @@
       <c r="P1" s="5"/>
       <c r="Q1" s="5"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:17">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -4004,7 +4379,7 @@
       <c r="P2" s="6"/>
       <c r="Q2" s="6"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:17">
       <c r="A3" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B3,D3)</f>
         <v>FactionRelation_Hero</v>
@@ -4034,7 +4409,7 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:17">
       <c r="A4" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B4,D4)</f>
         <v>FactionRelation_Faction2</v>
@@ -4064,7 +4439,7 @@
       </c>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:17">
       <c r="A5" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B5,D5)</f>
         <v>FactionRelation_Faction3</v>
@@ -4094,7 +4469,7 @@
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:17">
       <c r="A6" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B6,D6)</f>
         <v>FactionRelation_Faction4</v>
@@ -4122,43 +4497,43 @@
         <v>Hostile,Hostile,Hostile,Friendly</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:17">
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:17">
       <c r="D8" s="9"/>
       <c r="E8" s="9"/>
       <c r="J8" s="9"/>
       <c r="K8" s="9"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:17">
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="J9" s="9"/>
       <c r="K9" s="9"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:17">
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="9"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:17">
       <c r="D11" s="9"/>
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:17">
       <c r="D12" s="9"/>
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
       <c r="J12" s="9"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:17">
       <c r="D13" s="9"/>
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
@@ -4182,12 +4557,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BD492A1-6B8F-1440-9D54-6461F12B20A3}">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -4207,7 +4582,7 @@
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
@@ -4221,7 +4596,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10">
       <c r="A3" s="7" t="str">
         <f t="shared" ref="A3:A8" si="0">_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
         <v>Grade_Common</v>
@@ -4242,7 +4617,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10">
       <c r="A4" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Grade_Uncommon</v>
@@ -4265,7 +4640,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10">
       <c r="A5" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Grade_Rare</v>
@@ -4288,7 +4663,7 @@
       <c r="I5" s="9"/>
       <c r="J5" s="9"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10">
       <c r="A6" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Grade_Epic</v>
@@ -4311,7 +4686,7 @@
       <c r="I6" s="9"/>
       <c r="J6" s="9"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10">
       <c r="A7" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Grade_Unique</v>
@@ -4334,7 +4709,7 @@
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10">
       <c r="A8" s="7" t="str">
         <f t="shared" si="0"/>
         <v>Grade_Legend</v>
@@ -4361,17 +4736,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDE1ACEB-A93E-084F-8B48-EB95313F04DB}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="1" width="16.84375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.15234375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6">
       <c r="A1" s="7"/>
       <c r="B1" s="7" t="s">
         <v>2</v>
@@ -4389,7 +4764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6">
       <c r="A2" s="7"/>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
@@ -4403,7 +4778,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6">
       <c r="A3" s="7" t="str">
         <f>_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
         <v>SynergeBiome_Test</v>
@@ -4424,19 +4799,19 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6">
       <c r="A4" s="7"/>
       <c r="D4" s="9"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6">
       <c r="A5" s="7"/>
       <c r="D5" s="9"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6">
       <c r="A6" s="7"/>
       <c r="D6" s="9"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6">
       <c r="A7" s="7" t="str">
         <f t="shared" ref="A7" si="0">_xlfn.TEXTJOIN("_",TRUE,B7,C7)</f>
         <v/>
@@ -4444,7 +4819,7 @@
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6">
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
     </row>
@@ -4464,96 +4839,4 @@
     </ext>
   </extLst>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E95C1629-BD9D-564A-BFD4-EB36E5A37A98}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="11.15234375" defaultRowHeight="17.5" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="1" width="18.3046875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A1" s="7"/>
-      <c r="B1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3" s="7" t="str">
-        <f>_xlfn.TEXTJOIN("_",TRUE,B3,C3)</f>
-        <v>SynergeElement_Test</v>
-      </c>
-      <c r="B3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="C4" s="9"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="C5" s="9"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="C6" s="9"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B5FDDF60-689E-184E-934A-907BC1C56072}">
-          <x14:formula1>
-            <xm:f>Enum!$I$2:$I$1017</xm:f>
-          </x14:formula1>
-          <xm:sqref>B5:B6</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
-</worksheet>
 </file>
</xml_diff>